<commit_message>
Modificats Burndown Chart i presentació dilluns
</commit_message>
<xml_diff>
--- a/documents/Sprint4/Burndownchart4.xlsx
+++ b/documents/Sprint4/Burndownchart4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hyp3r\Desktop\Class\UAB\Sem2\ES\Sprints\GitHub\ES23UAB431-02\documents\Sprint4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E4EE99C-F215-4639-884D-B6E766D7492E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2385E9FF-5601-4EAC-9F21-BBF27C954417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -538,6 +538,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -548,9 +551,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -636,31 +636,31 @@
                   <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>26</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>26</c:v>
+                  <c:v>6</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>26</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>26</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>26</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>26</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>26</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>26</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>26</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1197,13 +1197,13 @@
     </row>
     <row r="2" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="25" t="s">
+      <c r="B2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="28"/>
       <c r="G2" s="4" t="s">
         <v>2</v>
       </c>
@@ -1235,11 +1235,11 @@
     </row>
     <row r="3" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
-      <c r="B3" s="28"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="30"/>
+      <c r="B3" s="29"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="30"/>
+      <c r="F3" s="31"/>
       <c r="G3" s="7"/>
       <c r="H3" s="8" t="s">
         <v>6</v>
@@ -1578,7 +1578,7 @@
       <c r="B12" s="16">
         <v>6</v>
       </c>
-      <c r="C12" s="31">
+      <c r="C12" s="25">
         <v>4</v>
       </c>
       <c r="D12" s="18">
@@ -1618,11 +1618,13 @@
       <c r="B13" s="16">
         <v>7</v>
       </c>
-      <c r="C13" s="17"/>
+      <c r="C13" s="17">
+        <v>10</v>
+      </c>
       <c r="D13" s="18"/>
       <c r="E13" s="21">
         <f>E12-C13</f>
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="F13" s="22">
         <f t="shared" ref="F13" si="6">F12-D13</f>
@@ -1654,11 +1656,13 @@
       <c r="B14" s="16">
         <v>8</v>
       </c>
-      <c r="C14" s="17"/>
+      <c r="C14" s="17">
+        <v>10</v>
+      </c>
       <c r="D14" s="18"/>
       <c r="E14" s="21">
         <f>E13-C14</f>
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="F14" s="22">
         <f t="shared" ref="F14" si="7">F13-D14</f>
@@ -1690,11 +1694,13 @@
       <c r="B15" s="16">
         <v>9</v>
       </c>
-      <c r="C15" s="17"/>
+      <c r="C15" s="17">
+        <v>4</v>
+      </c>
       <c r="D15" s="18"/>
       <c r="E15" s="21">
         <f t="shared" ref="E15:F15" si="8">E14-C15</f>
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="F15" s="22">
         <f t="shared" si="8"/>
@@ -1726,11 +1732,13 @@
       <c r="B16" s="16">
         <v>10</v>
       </c>
-      <c r="C16" s="17"/>
+      <c r="C16" s="17">
+        <v>2</v>
+      </c>
       <c r="D16" s="18"/>
       <c r="E16" s="21">
         <f t="shared" ref="E16:F16" si="9">E15-C16</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F16" s="22">
         <f t="shared" si="9"/>
@@ -1766,7 +1774,7 @@
       <c r="D17" s="18"/>
       <c r="E17" s="21">
         <f t="shared" ref="E17:F17" si="10">E16-C17</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F17" s="22">
         <f t="shared" si="10"/>
@@ -1802,7 +1810,7 @@
       <c r="D18" s="18"/>
       <c r="E18" s="21">
         <f t="shared" ref="E18:F18" si="11">E17-C18</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F18" s="22">
         <f t="shared" si="11"/>
@@ -1838,7 +1846,7 @@
       <c r="D19" s="18"/>
       <c r="E19" s="21">
         <f t="shared" ref="E19:F19" si="12">E18-C19</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F19" s="22">
         <f t="shared" si="12"/>
@@ -1874,7 +1882,7 @@
       <c r="D20" s="18"/>
       <c r="E20" s="21">
         <f t="shared" ref="E20:F20" si="13">E19-C20</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F20" s="22">
         <f t="shared" si="13"/>
@@ -1910,7 +1918,7 @@
       <c r="D21" s="18"/>
       <c r="E21" s="21">
         <f t="shared" ref="E21:F21" si="14">E20-C21</f>
-        <v>26</v>
+        <v>0</v>
       </c>
       <c r="F21" s="22">
         <f t="shared" si="14"/>

</xml_diff>

<commit_message>
Afegit 8. Modificar Disponibilitat
</commit_message>
<xml_diff>
--- a/documents/Sprint4/Burndownchart4.xlsx
+++ b/documents/Sprint4/Burndownchart4.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hyp3r\Desktop\Class\UAB\Sem2\ES\Sprints\GitHub\ES23UAB431-02\documents\Sprint4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2385E9FF-5601-4EAC-9F21-BBF27C954417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5EC45A-E853-4631-96B1-9EB9697786EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,10 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
-  <si>
-    <t>SIMPLE BURNDOWN CHART TEMPLATE</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>PROJECT TITLE</t>
   </si>
@@ -56,15 +53,6 @@
   </si>
   <si>
     <t>PROJECT ID</t>
-  </si>
-  <si>
-    <t>00/00/0000</t>
-  </si>
-  <si>
-    <t>1.0</t>
-  </si>
-  <si>
-    <t>PILOT-0628</t>
   </si>
   <si>
     <t>DAY / 
@@ -87,15 +75,27 @@
   <si>
     <t>BURNDOWN</t>
   </si>
+  <si>
+    <t>BURNDOWN CHART</t>
+  </si>
+  <si>
+    <t>Sprint 4: ES 2025/26</t>
+  </si>
+  <si>
+    <t>Martí Pagès Sánchez</t>
+  </si>
+  <si>
+    <t>2.0</t>
+  </si>
+  <si>
+    <t>ES25/26-431-02</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
-  </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -140,6 +140,19 @@
     <font>
       <u/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Century Gothic"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Century Gothic"/>
       <family val="2"/>
@@ -466,7 +479,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -487,15 +500,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -510,9 +514,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -551,6 +552,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="6" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="4" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="4" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -608,12 +624,63 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'BLANK - Simple Burndown Chart'!$B$6:$B$19</c:f>
+              <c:numCache>
+                <c:formatCode>d\-mmm</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>46167</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46168</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46169</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46170</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46171</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46172</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46173</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46174</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46175</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46176</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46177</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46178</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46179</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46180</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'BLANK - Simple Burndown Chart'!$E$6:$E$21</c:f>
+              <c:f>'BLANK - Simple Burndown Chart'!$E$6:$E$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>70</c:v>
                 </c:pt>
@@ -656,12 +723,6 @@
                 <c:pt idx="13">
                   <c:v>0</c:v>
                 </c:pt>
-                <c:pt idx="14">
-                  <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>0</c:v>
-                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
@@ -690,12 +751,63 @@
           <c:marker>
             <c:symbol val="none"/>
           </c:marker>
+          <c:cat>
+            <c:numRef>
+              <c:f>'BLANK - Simple Burndown Chart'!$B$6:$B$19</c:f>
+              <c:numCache>
+                <c:formatCode>d\-mmm</c:formatCode>
+                <c:ptCount val="14"/>
+                <c:pt idx="0">
+                  <c:v>46167</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>46168</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>46169</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>46170</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>46171</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>46172</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>46173</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>46174</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>46175</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>46176</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>46177</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>46178</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>46179</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>46180</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>'BLANK - Simple Burndown Chart'!$F$6:$F$21</c:f>
+              <c:f>'BLANK - Simple Burndown Chart'!$F$6:$F$19</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="16"/>
+                <c:ptCount val="14"/>
                 <c:pt idx="0">
                   <c:v>70</c:v>
                 </c:pt>
@@ -718,31 +830,25 @@
                   <c:v>26</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>26</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>26</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>26</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>26</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>26</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>26</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="14">
-                  <c:v>26</c:v>
-                </c:pt>
-                <c:pt idx="15">
-                  <c:v>26</c:v>
+                  <c:v>2</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -766,7 +872,7 @@
         <c:axId val="1725496515"/>
         <c:axId val="348616111"/>
       </c:lineChart>
-      <c:catAx>
+      <c:dateAx>
         <c:axId val="1725496515"/>
         <c:scaling>
           <c:orientation val="minMax"/>
@@ -791,7 +897,7 @@
           </c:tx>
           <c:overlay val="0"/>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="d\-mmm" sourceLinked="1"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -813,10 +919,9 @@
         <c:crossAx val="348616111"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
-        <c:lblAlgn val="ctr"/>
         <c:lblOffset val="100"/>
-        <c:noMultiLvlLbl val="1"/>
-      </c:catAx>
+        <c:baseTimeUnit val="days"/>
+      </c:dateAx>
       <c:valAx>
         <c:axId val="348616111"/>
         <c:scaling>
@@ -922,9 +1027,9 @@
   <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>6</xdr:col>
-      <xdr:colOff>57150</xdr:colOff>
+      <xdr:colOff>29441</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>781050</xdr:rowOff>
+      <xdr:rowOff>199159</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="5829300" cy="6248400"/>
     <xdr:graphicFrame macro="">
@@ -1155,7 +1260,7 @@
     <tabColor rgb="FFD6DCE4"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Z1000"/>
+  <dimension ref="A1:Z998"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.19921875" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3.3984375" customWidth="1"/>
@@ -1172,8 +1277,8 @@
   <sheetData>
     <row r="1" spans="1:26" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
-      <c r="B1" s="23" t="s">
-        <v>0</v>
+      <c r="B1" s="19" t="s">
+        <v>11</v>
       </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -1197,24 +1302,24 @@
     </row>
     <row r="2" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="22" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="28"/>
-      <c r="G2" s="4" t="s">
+      <c r="H2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="4" t="s">
+      <c r="J2" s="6" t="s">
         <v>4</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>5</v>
       </c>
       <c r="K2" s="3"/>
       <c r="L2" s="3"/>
@@ -1235,20 +1340,24 @@
     </row>
     <row r="3" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="8" t="s">
-        <v>6</v>
+      <c r="B3" s="25" t="s">
+        <v>12</v>
       </c>
-      <c r="I3" s="9" t="s">
-        <v>7</v>
+      <c r="C3" s="26"/>
+      <c r="D3" s="26"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="27"/>
+      <c r="G3" s="7" t="s">
+        <v>13</v>
       </c>
-      <c r="J3" s="10" t="s">
-        <v>8</v>
+      <c r="H3" s="29">
+        <v>46176</v>
+      </c>
+      <c r="I3" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="J3" s="31" t="s">
+        <v>15</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
@@ -1297,23 +1406,23 @@
     </row>
     <row r="5" spans="1:26" ht="69.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="C5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="11" t="s">
+      <c r="G5" s="12" t="s">
         <v>10</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" s="13" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="G5" s="15" t="s">
-        <v>14</v>
       </c>
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
@@ -1337,19 +1446,19 @@
     </row>
     <row r="6" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="16">
+      <c r="B6" s="28">
+        <v>46167</v>
+      </c>
+      <c r="C6" s="13">
         <v>0</v>
       </c>
-      <c r="C6" s="17">
+      <c r="D6" s="14">
         <v>0</v>
       </c>
-      <c r="D6" s="18">
-        <v>0</v>
-      </c>
-      <c r="E6" s="19">
+      <c r="E6" s="15">
         <v>70</v>
       </c>
-      <c r="F6" s="20">
+      <c r="F6" s="16">
         <v>70</v>
       </c>
       <c r="G6" s="1"/>
@@ -1375,20 +1484,20 @@
     </row>
     <row r="7" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="16">
-        <v>1</v>
+      <c r="B7" s="28">
+        <v>46168</v>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="13">
         <v>0</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="14">
         <v>0</v>
       </c>
-      <c r="E7" s="21">
+      <c r="E7" s="17">
         <f t="shared" ref="E7:F7" si="0">E6-C7</f>
         <v>70</v>
       </c>
-      <c r="F7" s="22">
+      <c r="F7" s="18">
         <f t="shared" si="0"/>
         <v>70</v>
       </c>
@@ -1415,20 +1524,20 @@
     </row>
     <row r="8" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="16">
+      <c r="B8" s="28">
+        <v>46169</v>
+      </c>
+      <c r="C8" s="13">
         <v>2</v>
       </c>
-      <c r="C8" s="17">
+      <c r="D8" s="14">
         <v>2</v>
       </c>
-      <c r="D8" s="18">
-        <v>2</v>
-      </c>
-      <c r="E8" s="21">
+      <c r="E8" s="17">
         <f t="shared" ref="E8" si="1">E7-C8</f>
         <v>68</v>
       </c>
-      <c r="F8" s="22">
+      <c r="F8" s="18">
         <f>F7-D8</f>
         <v>68</v>
       </c>
@@ -1455,20 +1564,20 @@
     </row>
     <row r="9" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="16">
-        <v>3</v>
+      <c r="B9" s="28">
+        <v>46170</v>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="13">
         <v>12</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="14">
         <v>8</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="17">
         <f t="shared" ref="E9" si="2">E8-C9</f>
         <v>56</v>
       </c>
-      <c r="F9" s="22">
+      <c r="F9" s="18">
         <f>F8-D9</f>
         <v>60</v>
       </c>
@@ -1495,20 +1604,20 @@
     </row>
     <row r="10" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="16">
-        <v>4</v>
+      <c r="B10" s="28">
+        <v>46171</v>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="13">
         <v>14</v>
       </c>
-      <c r="D10" s="24">
+      <c r="D10" s="20">
         <v>12</v>
       </c>
-      <c r="E10" s="21">
+      <c r="E10" s="17">
         <f t="shared" ref="E10:F10" si="3">E9-C10</f>
         <v>42</v>
       </c>
-      <c r="F10" s="22">
+      <c r="F10" s="18">
         <f t="shared" si="3"/>
         <v>48</v>
       </c>
@@ -1535,20 +1644,20 @@
     </row>
     <row r="11" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="16">
-        <v>5</v>
+      <c r="B11" s="28">
+        <v>46172</v>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="13">
         <v>12</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="14">
         <v>16</v>
       </c>
-      <c r="E11" s="21">
+      <c r="E11" s="17">
         <f t="shared" ref="E11:F11" si="4">E10-C11</f>
         <v>30</v>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="18">
         <f t="shared" si="4"/>
         <v>32</v>
       </c>
@@ -1575,20 +1684,20 @@
     </row>
     <row r="12" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="16">
+      <c r="B12" s="28">
+        <v>46173</v>
+      </c>
+      <c r="C12" s="21">
+        <v>4</v>
+      </c>
+      <c r="D12" s="14">
         <v>6</v>
       </c>
-      <c r="C12" s="25">
-        <v>4</v>
-      </c>
-      <c r="D12" s="18">
-        <v>6</v>
-      </c>
-      <c r="E12" s="21">
+      <c r="E12" s="17">
         <f t="shared" ref="E12:F12" si="5">E11-C12</f>
         <v>26</v>
       </c>
-      <c r="F12" s="22">
+      <c r="F12" s="18">
         <f t="shared" si="5"/>
         <v>26</v>
       </c>
@@ -1615,20 +1724,22 @@
     </row>
     <row r="13" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="16">
-        <v>7</v>
+      <c r="B13" s="28">
+        <v>46174</v>
       </c>
-      <c r="C13" s="17">
+      <c r="C13" s="13">
         <v>10</v>
       </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="21">
+      <c r="D13" s="14">
+        <v>4</v>
+      </c>
+      <c r="E13" s="17">
         <f>E12-C13</f>
         <v>16</v>
       </c>
-      <c r="F13" s="22">
+      <c r="F13" s="18">
         <f t="shared" ref="F13" si="6">F12-D13</f>
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="G13" s="1"/>
       <c r="H13" s="1"/>
@@ -1638,7 +1749,7 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
-      <c r="O13" s="1"/>
+      <c r="O13" s="32"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
@@ -1653,20 +1764,22 @@
     </row>
     <row r="14" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="16">
-        <v>8</v>
+      <c r="B14" s="28">
+        <v>46175</v>
       </c>
-      <c r="C14" s="17">
+      <c r="C14" s="13">
         <v>10</v>
       </c>
-      <c r="D14" s="18"/>
-      <c r="E14" s="21">
+      <c r="D14" s="14">
+        <v>6</v>
+      </c>
+      <c r="E14" s="17">
         <f>E13-C14</f>
         <v>6</v>
       </c>
-      <c r="F14" s="22">
+      <c r="F14" s="18">
         <f t="shared" ref="F14" si="7">F13-D14</f>
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
@@ -1691,20 +1804,22 @@
     </row>
     <row r="15" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="16">
-        <v>9</v>
+      <c r="B15" s="28">
+        <v>46176</v>
       </c>
-      <c r="C15" s="17">
+      <c r="C15" s="13">
         <v>4</v>
       </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="21">
+      <c r="D15" s="14">
+        <v>14</v>
+      </c>
+      <c r="E15" s="17">
         <f t="shared" ref="E15:F15" si="8">E14-C15</f>
         <v>2</v>
       </c>
-      <c r="F15" s="22">
+      <c r="F15" s="18">
         <f t="shared" si="8"/>
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -1729,20 +1844,20 @@
     </row>
     <row r="16" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="16">
-        <v>10</v>
+      <c r="B16" s="28">
+        <v>46177</v>
       </c>
-      <c r="C16" s="17">
+      <c r="C16" s="13">
         <v>2</v>
       </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="21">
+      <c r="D16" s="14"/>
+      <c r="E16" s="17">
         <f t="shared" ref="E16:F16" si="9">E15-C16</f>
         <v>0</v>
       </c>
-      <c r="F16" s="22">
+      <c r="F16" s="18">
         <f t="shared" si="9"/>
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -1767,18 +1882,18 @@
     </row>
     <row r="17" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="16">
-        <v>11</v>
+      <c r="B17" s="28">
+        <v>46178</v>
       </c>
-      <c r="C17" s="17"/>
-      <c r="D17" s="18"/>
-      <c r="E17" s="21">
+      <c r="C17" s="13"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="17">
         <f t="shared" ref="E17:F17" si="10">E16-C17</f>
         <v>0</v>
       </c>
-      <c r="F17" s="22">
+      <c r="F17" s="18">
         <f t="shared" si="10"/>
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -1803,18 +1918,18 @@
     </row>
     <row r="18" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="16">
-        <v>12</v>
+      <c r="B18" s="28">
+        <v>46179</v>
       </c>
-      <c r="C18" s="17"/>
-      <c r="D18" s="18"/>
-      <c r="E18" s="21">
+      <c r="C18" s="13"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="17">
         <f t="shared" ref="E18:F18" si="11">E17-C18</f>
         <v>0</v>
       </c>
-      <c r="F18" s="22">
+      <c r="F18" s="18">
         <f t="shared" si="11"/>
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -1839,18 +1954,18 @@
     </row>
     <row r="19" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="16">
-        <v>13</v>
+      <c r="B19" s="28">
+        <v>46180</v>
       </c>
-      <c r="C19" s="17"/>
-      <c r="D19" s="18"/>
-      <c r="E19" s="21">
+      <c r="C19" s="13"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="17">
         <f t="shared" ref="E19:F19" si="12">E18-C19</f>
         <v>0</v>
       </c>
-      <c r="F19" s="22">
+      <c r="F19" s="18">
         <f t="shared" si="12"/>
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
@@ -1873,21 +1988,13 @@
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
     </row>
-    <row r="20" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:26" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="16">
-        <v>14</v>
-      </c>
-      <c r="C20" s="17"/>
-      <c r="D20" s="18"/>
-      <c r="E20" s="21">
-        <f t="shared" ref="E20:F20" si="13">E19-C20</f>
-        <v>0</v>
-      </c>
-      <c r="F20" s="22">
-        <f t="shared" si="13"/>
-        <v>26</v>
-      </c>
+      <c r="B20" s="1"/>
+      <c r="C20" s="1"/>
+      <c r="D20" s="1"/>
+      <c r="E20" s="1"/>
+      <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
       <c r="I20" s="1"/>
@@ -1909,21 +2016,13 @@
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
     </row>
-    <row r="21" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="16">
-        <v>15</v>
-      </c>
-      <c r="C21" s="17"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="21">
-        <f t="shared" ref="E21:F21" si="14">E20-C21</f>
-        <v>0</v>
-      </c>
-      <c r="F21" s="22">
-        <f t="shared" si="14"/>
-        <v>26</v>
-      </c>
+      <c r="B21" s="1"/>
+      <c r="C21" s="1"/>
+      <c r="D21" s="1"/>
+      <c r="E21" s="1"/>
+      <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
       <c r="I21" s="1"/>
@@ -1945,7 +2044,7 @@
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
     </row>
-    <row r="22" spans="1:26" ht="58.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
@@ -1973,18 +2072,18 @@
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
     </row>
-    <row r="23" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
-      <c r="F23" s="1"/>
+    <row r="23" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
       <c r="I23" s="1"/>
-      <c r="J23" s="1"/>
-      <c r="K23" s="1"/>
+      <c r="J23" s="2"/>
+      <c r="K23" s="2"/>
       <c r="L23" s="1"/>
       <c r="M23" s="1"/>
       <c r="N23" s="1"/>
@@ -2001,18 +2100,18 @@
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
     </row>
-    <row r="24" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
-      <c r="F24" s="1"/>
+    <row r="24" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
-      <c r="J24" s="1"/>
-      <c r="K24" s="1"/>
+      <c r="J24" s="2"/>
+      <c r="K24" s="2"/>
       <c r="L24" s="1"/>
       <c r="M24" s="1"/>
       <c r="N24" s="1"/>
@@ -7490,17 +7589,17 @@
       <c r="Z219" s="1"/>
     </row>
     <row r="220" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A220" s="2"/>
-      <c r="B220" s="2"/>
-      <c r="C220" s="2"/>
-      <c r="D220" s="2"/>
-      <c r="E220" s="2"/>
-      <c r="F220" s="2"/>
+      <c r="A220" s="1"/>
+      <c r="B220" s="1"/>
+      <c r="C220" s="1"/>
+      <c r="D220" s="1"/>
+      <c r="E220" s="1"/>
+      <c r="F220" s="1"/>
       <c r="G220" s="1"/>
       <c r="H220" s="1"/>
       <c r="I220" s="1"/>
-      <c r="J220" s="2"/>
-      <c r="K220" s="2"/>
+      <c r="J220" s="1"/>
+      <c r="K220" s="1"/>
       <c r="L220" s="1"/>
       <c r="M220" s="1"/>
       <c r="N220" s="1"/>
@@ -7518,17 +7617,17 @@
       <c r="Z220" s="1"/>
     </row>
     <row r="221" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A221" s="2"/>
-      <c r="B221" s="2"/>
-      <c r="C221" s="2"/>
-      <c r="D221" s="2"/>
-      <c r="E221" s="2"/>
-      <c r="F221" s="2"/>
+      <c r="A221" s="1"/>
+      <c r="B221" s="1"/>
+      <c r="C221" s="1"/>
+      <c r="D221" s="1"/>
+      <c r="E221" s="1"/>
+      <c r="F221" s="1"/>
       <c r="G221" s="1"/>
       <c r="H221" s="1"/>
       <c r="I221" s="1"/>
-      <c r="J221" s="2"/>
-      <c r="K221" s="2"/>
+      <c r="J221" s="1"/>
+      <c r="K221" s="1"/>
       <c r="L221" s="1"/>
       <c r="M221" s="1"/>
       <c r="N221" s="1"/>
@@ -29301,62 +29400,6 @@
       <c r="Y998" s="1"/>
       <c r="Z998" s="1"/>
     </row>
-    <row r="999" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A999" s="1"/>
-      <c r="B999" s="1"/>
-      <c r="C999" s="1"/>
-      <c r="D999" s="1"/>
-      <c r="E999" s="1"/>
-      <c r="F999" s="1"/>
-      <c r="G999" s="1"/>
-      <c r="H999" s="1"/>
-      <c r="I999" s="1"/>
-      <c r="J999" s="1"/>
-      <c r="K999" s="1"/>
-      <c r="L999" s="1"/>
-      <c r="M999" s="1"/>
-      <c r="N999" s="1"/>
-      <c r="O999" s="1"/>
-      <c r="P999" s="1"/>
-      <c r="Q999" s="1"/>
-      <c r="R999" s="1"/>
-      <c r="S999" s="1"/>
-      <c r="T999" s="1"/>
-      <c r="U999" s="1"/>
-      <c r="V999" s="1"/>
-      <c r="W999" s="1"/>
-      <c r="X999" s="1"/>
-      <c r="Y999" s="1"/>
-      <c r="Z999" s="1"/>
-    </row>
-    <row r="1000" spans="1:26" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1000" s="1"/>
-      <c r="B1000" s="1"/>
-      <c r="C1000" s="1"/>
-      <c r="D1000" s="1"/>
-      <c r="E1000" s="1"/>
-      <c r="F1000" s="1"/>
-      <c r="G1000" s="1"/>
-      <c r="H1000" s="1"/>
-      <c r="I1000" s="1"/>
-      <c r="J1000" s="1"/>
-      <c r="K1000" s="1"/>
-      <c r="L1000" s="1"/>
-      <c r="M1000" s="1"/>
-      <c r="N1000" s="1"/>
-      <c r="O1000" s="1"/>
-      <c r="P1000" s="1"/>
-      <c r="Q1000" s="1"/>
-      <c r="R1000" s="1"/>
-      <c r="S1000" s="1"/>
-      <c r="T1000" s="1"/>
-      <c r="U1000" s="1"/>
-      <c r="V1000" s="1"/>
-      <c r="W1000" s="1"/>
-      <c r="X1000" s="1"/>
-      <c r="Y1000" s="1"/>
-      <c r="Z1000" s="1"/>
-    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B2:F2"/>

</xml_diff>

<commit_message>
Actualitzats 1., prese i burndown
</commit_message>
<xml_diff>
--- a/documents/Sprint4/Burndownchart4.xlsx
+++ b/documents/Sprint4/Burndownchart4.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hyp3r\Desktop\Class\UAB\Sem2\ES\Sprints\GitHub\ES23UAB431-02\documents\Sprint4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA5EC45A-E853-4631-96B1-9EB9697786EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83AC21AA-BB2D-47DD-AD8C-78FC0F0B52AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -85,10 +85,10 @@
     <t>Martí Pagès Sánchez</t>
   </si>
   <si>
-    <t>2.0</t>
+    <t>ES25/26-431-02</t>
   </si>
   <si>
-    <t>ES25/26-431-02</t>
+    <t>3.0</t>
   </si>
 </sst>
 </file>
@@ -542,16 +542,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="16" fontId="6" fillId="8" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -567,6 +557,16 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -839,16 +839,16 @@
                   <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>2</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>2</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>2</c:v>
+                  <c:v>1</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>2</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1302,13 +1302,13 @@
     </row>
     <row r="2" spans="1:26" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3"/>
-      <c r="B2" s="22" t="s">
+      <c r="B2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="23"/>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="24"/>
+      <c r="C2" s="28"/>
+      <c r="D2" s="28"/>
+      <c r="E2" s="28"/>
+      <c r="F2" s="29"/>
       <c r="G2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1340,24 +1340,24 @@
     </row>
     <row r="3" spans="1:26" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3"/>
-      <c r="B3" s="25" t="s">
+      <c r="B3" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="26"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="27"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="32"/>
       <c r="G3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H3" s="29">
+      <c r="H3" s="23">
         <v>46176</v>
       </c>
-      <c r="I3" s="30" t="s">
+      <c r="I3" s="24" t="s">
+        <v>15</v>
+      </c>
+      <c r="J3" s="25" t="s">
         <v>14</v>
-      </c>
-      <c r="J3" s="31" t="s">
-        <v>15</v>
       </c>
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
@@ -1446,7 +1446,7 @@
     </row>
     <row r="6" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="28">
+      <c r="B6" s="22">
         <v>46167</v>
       </c>
       <c r="C6" s="13">
@@ -1484,7 +1484,7 @@
     </row>
     <row r="7" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="28">
+      <c r="B7" s="22">
         <v>46168</v>
       </c>
       <c r="C7" s="13">
@@ -1524,7 +1524,7 @@
     </row>
     <row r="8" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="28">
+      <c r="B8" s="22">
         <v>46169</v>
       </c>
       <c r="C8" s="13">
@@ -1564,7 +1564,7 @@
     </row>
     <row r="9" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="28">
+      <c r="B9" s="22">
         <v>46170</v>
       </c>
       <c r="C9" s="13">
@@ -1604,7 +1604,7 @@
     </row>
     <row r="10" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="28">
+      <c r="B10" s="22">
         <v>46171</v>
       </c>
       <c r="C10" s="13">
@@ -1631,7 +1631,7 @@
       <c r="N10" s="1"/>
       <c r="O10" s="1"/>
       <c r="P10" s="1"/>
-      <c r="Q10" s="1"/>
+      <c r="Q10" s="26"/>
       <c r="R10" s="1"/>
       <c r="S10" s="1"/>
       <c r="T10" s="1"/>
@@ -1644,7 +1644,7 @@
     </row>
     <row r="11" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="28">
+      <c r="B11" s="22">
         <v>46172</v>
       </c>
       <c r="C11" s="13">
@@ -1684,7 +1684,7 @@
     </row>
     <row r="12" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="28">
+      <c r="B12" s="22">
         <v>46173</v>
       </c>
       <c r="C12" s="21">
@@ -1724,7 +1724,7 @@
     </row>
     <row r="13" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="28">
+      <c r="B13" s="22">
         <v>46174</v>
       </c>
       <c r="C13" s="13">
@@ -1749,7 +1749,7 @@
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
-      <c r="O13" s="32"/>
+      <c r="O13" s="26"/>
       <c r="P13" s="1"/>
       <c r="Q13" s="1"/>
       <c r="R13" s="1"/>
@@ -1764,7 +1764,7 @@
     </row>
     <row r="14" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="28">
+      <c r="B14" s="22">
         <v>46175</v>
       </c>
       <c r="C14" s="13">
@@ -1804,7 +1804,7 @@
     </row>
     <row r="15" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="28">
+      <c r="B15" s="22">
         <v>46176</v>
       </c>
       <c r="C15" s="13">
@@ -1844,20 +1844,22 @@
     </row>
     <row r="16" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="28">
+      <c r="B16" s="22">
         <v>46177</v>
       </c>
       <c r="C16" s="13">
         <v>2</v>
       </c>
-      <c r="D16" s="14"/>
+      <c r="D16" s="14">
+        <v>1</v>
+      </c>
       <c r="E16" s="17">
         <f t="shared" ref="E16:F16" si="9">E15-C16</f>
         <v>0</v>
       </c>
       <c r="F16" s="18">
         <f t="shared" si="9"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -1882,18 +1884,22 @@
     </row>
     <row r="17" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="28">
+      <c r="B17" s="22">
         <v>46178</v>
       </c>
-      <c r="C17" s="13"/>
-      <c r="D17" s="14"/>
+      <c r="C17" s="13">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14">
+        <v>0</v>
+      </c>
       <c r="E17" s="17">
         <f t="shared" ref="E17:F17" si="10">E16-C17</f>
         <v>0</v>
       </c>
       <c r="F17" s="18">
         <f t="shared" si="10"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -1918,18 +1924,22 @@
     </row>
     <row r="18" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="28">
+      <c r="B18" s="22">
         <v>46179</v>
       </c>
-      <c r="C18" s="13"/>
-      <c r="D18" s="14"/>
+      <c r="C18" s="13">
+        <v>0</v>
+      </c>
+      <c r="D18" s="14">
+        <v>0</v>
+      </c>
       <c r="E18" s="17">
         <f t="shared" ref="E18:F18" si="11">E17-C18</f>
         <v>0</v>
       </c>
       <c r="F18" s="18">
         <f t="shared" si="11"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -1954,18 +1964,22 @@
     </row>
     <row r="19" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="28">
+      <c r="B19" s="22">
         <v>46180</v>
       </c>
-      <c r="C19" s="13"/>
-      <c r="D19" s="14"/>
+      <c r="C19" s="13">
+        <v>0</v>
+      </c>
+      <c r="D19" s="14">
+        <v>1</v>
+      </c>
       <c r="E19" s="17">
         <f t="shared" ref="E19:F19" si="12">E18-C19</f>
         <v>0</v>
       </c>
       <c r="F19" s="18">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>

</xml_diff>